<commit_message>
Updated Playwright automation scripts
</commit_message>
<xml_diff>
--- a/EASAAutomationWorkFlows/data/easa-data.xlsx
+++ b/EASAAutomationWorkFlows/data/easa-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinee\PlaywrightBolt\EASAApplicationProcess\EASAAutomationWorkFlows\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE52B919-FF1D-46E1-BB98-6D9B7270A009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1852AD56-FA0E-4A6F-A296-587DDCC0BF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Approvals" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="46">
   <si>
     <t>Variant</t>
   </si>
@@ -97,12 +97,6 @@
     <t>Audit</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
     <t>Rahul Toky</t>
   </si>
   <si>
@@ -161,6 +155,24 @@
   </si>
   <si>
     <t>AVIATION HOUSE (street3)</t>
+  </si>
+  <si>
+    <t>StakeHolderName</t>
+  </si>
+  <si>
+    <t>StakeHolderRole</t>
+  </si>
+  <si>
+    <t>Team Leader</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Monday 4 May</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Friday 1 May</t>
+  </si>
+  <si>
+    <t>s</t>
   </si>
 </sst>
 </file>
@@ -543,7 +555,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -556,7 +568,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -565,9 +577,11 @@
     <col min="5" max="5" width="24.77734375" customWidth="1"/>
     <col min="6" max="6" width="17.109375" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" customWidth="1"/>
+    <col min="8" max="8" width="17.77734375" customWidth="1"/>
+    <col min="9" max="9" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -578,63 +592,81 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
         <v>31</v>
       </c>
-      <c r="E1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>33</v>
       </c>
-      <c r="G1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
         <v>38</v>
       </c>
-      <c r="C2" t="s">
-        <v>40</v>
-      </c>
       <c r="D2" s="1">
-        <v>46029</v>
+        <v>46027</v>
       </c>
       <c r="E2" s="1">
         <v>46030</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="1">
-        <v>46029</v>
+        <v>46027</v>
       </c>
       <c r="E3" s="1">
         <v>46030</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -645,21 +677,27 @@
         <v>10</v>
       </c>
       <c r="D4" s="1">
-        <v>46029</v>
+        <v>46027</v>
       </c>
       <c r="E4" s="1">
         <v>46030</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -671,12 +709,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" customWidth="1"/>
     <col min="5" max="5" width="17.109375" customWidth="1"/>
     <col min="6" max="6" width="24.33203125" customWidth="1"/>
     <col min="7" max="7" width="18.5546875" customWidth="1"/>
@@ -702,7 +740,7 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G1" t="s">
         <v>15</v>
@@ -725,28 +763,28 @@
         <v>19</v>
       </c>
       <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>24</v>
-      </c>
-      <c r="I2" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -757,28 +795,28 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
       <c r="J3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -789,28 +827,33 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
         <v>21</v>
       </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
       <c r="J4" t="s">
-        <v>41</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F21" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>